<commit_message>
learned pandas shapes, columns and filtering
</commit_message>
<xml_diff>
--- a/output_excel.xlsx
+++ b/output_excel.xlsx
@@ -451,11 +451,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Raj</t>
+          <t>Alyssa</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>21</v>
+        <v>2382</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>

</xml_diff>